<commit_message>
Drop _data sheet, fix dept switching jitter, add duration recalc, UI polish
- Remove _data JSON sheet from Excel read/write; always use cell-by-cell parsing
- Clean up legacy _data sheets on save
- Read meeting ratings directly from Excel cells B192:B201
- Show parse error page when Excel file can't be rendered
- Fix department sidebar double-load by using history.replaceState
- Recalculate duration live when start/end time inputs change
- Replace About page back button with X close button
- Reorder settings menu: group folder and logo actions with divider
</commit_message>
<xml_diff>
--- a/src/blank.xlsx
+++ b/src/blank.xlsx
@@ -9,9 +9,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MohammadAdib\Documents\GitHub\CompanyTools\src\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{595F0BC8-939C-4EAB-B0D5-95EA80A9C2B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F31A0A79-E2DF-49D0-9056-532A018587C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1116" yWindow="1116" windowWidth="23040" windowHeight="13560" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="768" yWindow="768" windowWidth="23040" windowHeight="13560" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="L10 Meeting" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="105">
   <si>
     <t>Team:</t>
   </si>
@@ -317,24 +317,6 @@
     <t>Wk 11</t>
   </si>
   <si>
-    <t>Measurable 5</t>
-  </si>
-  <si>
-    <t>Measurable 6</t>
-  </si>
-  <si>
-    <t>Measurable 7</t>
-  </si>
-  <si>
-    <t>Measurable 8</t>
-  </si>
-  <si>
-    <t>Measurable 9</t>
-  </si>
-  <si>
-    <t>Measurable 10</t>
-  </si>
-  <si>
     <t xml:space="preserve">  Tip: Use conditional formatting on weekly cells — orange fill for Off Track, white for On Track.</t>
   </si>
   <si>
@@ -347,27 +329,6 @@
     <t>#</t>
   </si>
   <si>
-    <t>OKR 1</t>
-  </si>
-  <si>
-    <t>OKR 2</t>
-  </si>
-  <si>
-    <t>OKR 3</t>
-  </si>
-  <si>
-    <t>OKR 4</t>
-  </si>
-  <si>
-    <t>OKR 5</t>
-  </si>
-  <si>
-    <t>OKR 6</t>
-  </si>
-  <si>
-    <t>OKR 7</t>
-  </si>
-  <si>
     <t xml:space="preserve">  KEY RESULTS  —  Break down each OKR into measurable outcomes</t>
   </si>
   <si>
@@ -384,27 +345,6 @@
   </si>
   <si>
     <t xml:space="preserve">  OKR #3  —  Key Results</t>
-  </si>
-  <si>
-    <t>Measurable 1</t>
-  </si>
-  <si>
-    <t>Measurable 2</t>
-  </si>
-  <si>
-    <t>Measurable 3</t>
-  </si>
-  <si>
-    <t>Measurable 4</t>
-  </si>
-  <si>
-    <t>OKR 8</t>
-  </si>
-  <si>
-    <t>OKR 9</t>
-  </si>
-  <si>
-    <t>OKR 10</t>
   </si>
   <si>
     <t>LEVEL 10 MEETING</t>
@@ -689,48 +629,29 @@
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="14" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="13" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -740,6 +661,25 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="14" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1071,8 +1011,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="33.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="33" t="s">
-        <v>122</v>
+      <c r="A1" s="16" t="s">
+        <v>102</v>
       </c>
       <c r="B1" s="17"/>
       <c r="C1" s="17"/>
@@ -1084,36 +1024,36 @@
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="27"/>
+      <c r="B2" s="21"/>
       <c r="C2" s="18"/>
       <c r="D2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="27"/>
+      <c r="E2" s="21"/>
       <c r="F2" s="18"/>
     </row>
     <row r="3" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="27"/>
+      <c r="B3" s="21"/>
       <c r="C3" s="18"/>
       <c r="D3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="27"/>
+      <c r="E3" s="21"/>
       <c r="F3" s="18"/>
     </row>
     <row r="4" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="27"/>
+      <c r="B4" s="21"/>
       <c r="C4" s="18"/>
       <c r="D4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="27"/>
+      <c r="E4" s="21"/>
       <c r="F4" s="18"/>
     </row>
     <row r="5" spans="1:6" ht="8.1" customHeight="1" x14ac:dyDescent="0.3">
@@ -1128,16 +1068,16 @@
       <c r="A6" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="20"/>
-      <c r="C6" s="20"/>
-      <c r="D6" s="20"/>
-      <c r="E6" s="21"/>
+      <c r="B6" s="24"/>
+      <c r="C6" s="24"/>
+      <c r="D6" s="24"/>
+      <c r="E6" s="25"/>
       <c r="F6" s="14" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="22" t="s">
+      <c r="A7" s="26" t="s">
         <v>8</v>
       </c>
       <c r="B7" s="17"/>
@@ -1147,24 +1087,24 @@
       <c r="F7" s="18"/>
     </row>
     <row r="8" spans="1:6" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="34" t="s">
+      <c r="A8" s="27" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="35"/>
-      <c r="C8" s="35"/>
-      <c r="D8" s="35"/>
-      <c r="E8" s="35"/>
-      <c r="F8" s="36"/>
+      <c r="B8" s="28"/>
+      <c r="C8" s="28"/>
+      <c r="D8" s="28"/>
+      <c r="E8" s="28"/>
+      <c r="F8" s="29"/>
     </row>
     <row r="9" spans="1:6" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="34" t="s">
+      <c r="A9" s="27" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="35"/>
-      <c r="C9" s="35"/>
-      <c r="D9" s="35"/>
-      <c r="E9" s="35"/>
-      <c r="F9" s="36"/>
+      <c r="B9" s="28"/>
+      <c r="C9" s="28"/>
+      <c r="D9" s="28"/>
+      <c r="E9" s="28"/>
+      <c r="F9" s="29"/>
     </row>
     <row r="10" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4"/>
@@ -1178,16 +1118,16 @@
       <c r="A11" s="23" t="s">
         <v>11</v>
       </c>
-      <c r="B11" s="20"/>
-      <c r="C11" s="20"/>
-      <c r="D11" s="20"/>
-      <c r="E11" s="21"/>
+      <c r="B11" s="24"/>
+      <c r="C11" s="24"/>
+      <c r="D11" s="24"/>
+      <c r="E11" s="25"/>
       <c r="F11" s="14" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="22" t="s">
+      <c r="A12" s="26" t="s">
         <v>12</v>
       </c>
       <c r="B12" s="17"/>
@@ -1217,9 +1157,9 @@
       </c>
     </row>
     <row r="14" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="2" t="str">
+      <c r="A14" s="2">
         <f>Scorecard!A4</f>
-        <v>Measurable 1</v>
+        <v>0</v>
       </c>
       <c r="B14" s="2"/>
       <c r="C14" s="3"/>
@@ -1228,9 +1168,9 @@
       <c r="F14" s="3"/>
     </row>
     <row r="15" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="8" t="str">
+      <c r="A15" s="8">
         <f>Scorecard!A5</f>
-        <v>Measurable 2</v>
+        <v>0</v>
       </c>
       <c r="B15" s="8"/>
       <c r="C15" s="9"/>
@@ -1239,9 +1179,9 @@
       <c r="F15" s="9"/>
     </row>
     <row r="16" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="2" t="str">
+      <c r="A16" s="2">
         <f>Scorecard!A6</f>
-        <v>Measurable 3</v>
+        <v>0</v>
       </c>
       <c r="B16" s="2"/>
       <c r="C16" s="3"/>
@@ -1250,9 +1190,9 @@
       <c r="F16" s="3"/>
     </row>
     <row r="17" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="8" t="str">
+      <c r="A17" s="8">
         <f>Scorecard!A7</f>
-        <v>Measurable 4</v>
+        <v>0</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="9"/>
@@ -1261,9 +1201,9 @@
       <c r="F17" s="9"/>
     </row>
     <row r="18" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="2" t="str">
+      <c r="A18" s="2">
         <f>Scorecard!A8</f>
-        <v>Measurable 5</v>
+        <v>0</v>
       </c>
       <c r="B18" s="2"/>
       <c r="C18" s="3"/>
@@ -1272,9 +1212,9 @@
       <c r="F18" s="3"/>
     </row>
     <row r="19" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="8" t="str">
+      <c r="A19" s="8">
         <f>Scorecard!A9</f>
-        <v>Measurable 6</v>
+        <v>0</v>
       </c>
       <c r="B19" s="8"/>
       <c r="C19" s="9"/>
@@ -1283,9 +1223,9 @@
       <c r="F19" s="9"/>
     </row>
     <row r="20" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="2" t="str">
+      <c r="A20" s="2">
         <f>Scorecard!A10</f>
-        <v>Measurable 7</v>
+        <v>0</v>
       </c>
       <c r="B20" s="2"/>
       <c r="C20" s="3"/>
@@ -1294,7 +1234,7 @@
       <c r="F20" s="3"/>
     </row>
     <row r="21" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="28" t="s">
+      <c r="A21" s="35" t="s">
         <v>19</v>
       </c>
       <c r="B21" s="17"/>
@@ -1315,16 +1255,16 @@
       <c r="A23" s="23" t="s">
         <v>20</v>
       </c>
-      <c r="B23" s="20"/>
-      <c r="C23" s="20"/>
-      <c r="D23" s="20"/>
-      <c r="E23" s="21"/>
+      <c r="B23" s="24"/>
+      <c r="C23" s="24"/>
+      <c r="D23" s="24"/>
+      <c r="E23" s="25"/>
       <c r="F23" s="14" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="22" t="s">
+      <c r="A24" s="26" t="s">
         <v>21</v>
       </c>
       <c r="B24" s="17"/>
@@ -1354,9 +1294,9 @@
       </c>
     </row>
     <row r="26" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="2" t="str">
+      <c r="A26" s="2">
         <f>OKRs!B5</f>
-        <v>OKR 1</v>
+        <v>0</v>
       </c>
       <c r="B26" s="2"/>
       <c r="C26" s="3"/>
@@ -1365,9 +1305,9 @@
       <c r="F26" s="3"/>
     </row>
     <row r="27" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="2" t="str">
+      <c r="A27" s="2">
         <f>OKRs!B6</f>
-        <v>OKR 2</v>
+        <v>0</v>
       </c>
       <c r="B27" s="8"/>
       <c r="C27" s="9"/>
@@ -1376,9 +1316,9 @@
       <c r="F27" s="9"/>
     </row>
     <row r="28" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="2" t="str">
+      <c r="A28" s="2">
         <f>OKRs!B7</f>
-        <v>OKR 3</v>
+        <v>0</v>
       </c>
       <c r="B28" s="2"/>
       <c r="C28" s="3"/>
@@ -1387,9 +1327,9 @@
       <c r="F28" s="3"/>
     </row>
     <row r="29" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="2" t="str">
+      <c r="A29" s="2">
         <f>OKRs!B8</f>
-        <v>OKR 4</v>
+        <v>0</v>
       </c>
       <c r="B29" s="8"/>
       <c r="C29" s="9"/>
@@ -1398,9 +1338,9 @@
       <c r="F29" s="9"/>
     </row>
     <row r="30" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="2" t="str">
+      <c r="A30" s="2">
         <f>OKRs!B9</f>
-        <v>OKR 5</v>
+        <v>0</v>
       </c>
       <c r="B30" s="2"/>
       <c r="C30" s="3"/>
@@ -1409,9 +1349,9 @@
       <c r="F30" s="3"/>
     </row>
     <row r="31" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="2" t="str">
+      <c r="A31" s="2">
         <f>OKRs!B10</f>
-        <v>OKR 6</v>
+        <v>0</v>
       </c>
       <c r="B31" s="8"/>
       <c r="C31" s="9"/>
@@ -1420,7 +1360,7 @@
       <c r="F31" s="9"/>
     </row>
     <row r="32" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="28" t="s">
+      <c r="A32" s="35" t="s">
         <v>25</v>
       </c>
       <c r="B32" s="17"/>
@@ -1441,16 +1381,16 @@
       <c r="A34" s="23" t="s">
         <v>26</v>
       </c>
-      <c r="B34" s="20"/>
-      <c r="C34" s="20"/>
-      <c r="D34" s="20"/>
-      <c r="E34" s="21"/>
+      <c r="B34" s="24"/>
+      <c r="C34" s="24"/>
+      <c r="D34" s="24"/>
+      <c r="E34" s="25"/>
       <c r="F34" s="14" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="35" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="22" t="s">
+      <c r="A35" s="26" t="s">
         <v>27</v>
       </c>
       <c r="B35" s="17"/>
@@ -1539,16 +1479,16 @@
       <c r="A44" s="23" t="s">
         <v>33</v>
       </c>
-      <c r="B44" s="20"/>
-      <c r="C44" s="20"/>
-      <c r="D44" s="20"/>
-      <c r="E44" s="21"/>
+      <c r="B44" s="24"/>
+      <c r="C44" s="24"/>
+      <c r="D44" s="24"/>
+      <c r="E44" s="25"/>
       <c r="F44" s="14" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="45" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="22" t="s">
+      <c r="A45" s="26" t="s">
         <v>34</v>
       </c>
       <c r="B45" s="17"/>
@@ -1634,20 +1574,20 @@
       <c r="F53" s="3"/>
     </row>
     <row r="54" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="29" t="s">
+      <c r="A54" s="20" t="s">
         <v>36</v>
       </c>
       <c r="B54" s="17"/>
       <c r="C54" s="17"/>
       <c r="D54" s="18"/>
-      <c r="E54" s="26" t="str">
+      <c r="E54" s="36" t="str">
         <f>COUNTIF(D47:D53,"✅ Done")&amp;" / 7 done"</f>
         <v>0 / 7 done</v>
       </c>
       <c r="F54" s="18"/>
     </row>
     <row r="55" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="28" t="s">
+      <c r="A55" s="35" t="s">
         <v>37</v>
       </c>
       <c r="B55" s="17"/>
@@ -1668,16 +1608,16 @@
       <c r="A57" s="23" t="s">
         <v>38</v>
       </c>
-      <c r="B57" s="20"/>
-      <c r="C57" s="20"/>
-      <c r="D57" s="20"/>
-      <c r="E57" s="21"/>
+      <c r="B57" s="24"/>
+      <c r="C57" s="24"/>
+      <c r="D57" s="24"/>
+      <c r="E57" s="25"/>
       <c r="F57" s="14" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="58" spans="1:6" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="25" t="s">
+      <c r="A58" s="30" t="s">
         <v>40</v>
       </c>
       <c r="B58" s="17"/>
@@ -1835,17 +1775,17 @@
       <c r="F75" s="4"/>
     </row>
     <row r="76" spans="1:6" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A76" s="19" t="s">
+      <c r="A76" s="33" t="s">
         <v>46</v>
       </c>
-      <c r="B76" s="20"/>
-      <c r="C76" s="20"/>
-      <c r="D76" s="20"/>
-      <c r="E76" s="20"/>
-      <c r="F76" s="21"/>
+      <c r="B76" s="24"/>
+      <c r="C76" s="24"/>
+      <c r="D76" s="24"/>
+      <c r="E76" s="24"/>
+      <c r="F76" s="25"/>
     </row>
     <row r="77" spans="1:6" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A77" s="24" t="s">
+      <c r="A77" s="22" t="s">
         <v>47</v>
       </c>
       <c r="B77" s="17"/>
@@ -1858,7 +1798,7 @@
       <c r="A78" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="B78" s="16" t="s">
+      <c r="B78" s="19" t="s">
         <v>49</v>
       </c>
       <c r="C78" s="17"/>
@@ -1870,7 +1810,7 @@
       <c r="A79" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="B79" s="16" t="s">
+      <c r="B79" s="19" t="s">
         <v>51</v>
       </c>
       <c r="C79" s="17"/>
@@ -1882,7 +1822,7 @@
       <c r="A80" s="12" t="s">
         <v>52</v>
       </c>
-      <c r="B80" s="16" t="s">
+      <c r="B80" s="19" t="s">
         <v>53</v>
       </c>
       <c r="C80" s="17"/>
@@ -1943,7 +1883,7 @@
       <c r="F85" s="4"/>
     </row>
     <row r="86" spans="1:6" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A86" s="24" t="s">
+      <c r="A86" s="22" t="s">
         <v>55</v>
       </c>
       <c r="B86" s="17"/>
@@ -1956,7 +1896,7 @@
       <c r="A87" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="B87" s="16" t="s">
+      <c r="B87" s="19" t="s">
         <v>49</v>
       </c>
       <c r="C87" s="17"/>
@@ -1968,7 +1908,7 @@
       <c r="A88" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="B88" s="16" t="s">
+      <c r="B88" s="19" t="s">
         <v>51</v>
       </c>
       <c r="C88" s="17"/>
@@ -1980,7 +1920,7 @@
       <c r="A89" s="12" t="s">
         <v>52</v>
       </c>
-      <c r="B89" s="16" t="s">
+      <c r="B89" s="19" t="s">
         <v>53</v>
       </c>
       <c r="C89" s="17"/>
@@ -2041,7 +1981,7 @@
       <c r="F94" s="4"/>
     </row>
     <row r="95" spans="1:6" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A95" s="24" t="s">
+      <c r="A95" s="22" t="s">
         <v>56</v>
       </c>
       <c r="B95" s="17"/>
@@ -2054,7 +1994,7 @@
       <c r="A96" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="B96" s="16" t="s">
+      <c r="B96" s="19" t="s">
         <v>49</v>
       </c>
       <c r="C96" s="17"/>
@@ -2066,7 +2006,7 @@
       <c r="A97" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="B97" s="16" t="s">
+      <c r="B97" s="19" t="s">
         <v>51</v>
       </c>
       <c r="C97" s="17"/>
@@ -2078,7 +2018,7 @@
       <c r="A98" s="12" t="s">
         <v>52</v>
       </c>
-      <c r="B98" s="16" t="s">
+      <c r="B98" s="19" t="s">
         <v>53</v>
       </c>
       <c r="C98" s="17"/>
@@ -2139,7 +2079,7 @@
       <c r="F103" s="4"/>
     </row>
     <row r="104" spans="1:6" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A104" s="24" t="s">
+      <c r="A104" s="22" t="s">
         <v>57</v>
       </c>
       <c r="B104" s="17"/>
@@ -2152,7 +2092,7 @@
       <c r="A105" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="B105" s="16" t="s">
+      <c r="B105" s="19" t="s">
         <v>49</v>
       </c>
       <c r="C105" s="17"/>
@@ -2164,7 +2104,7 @@
       <c r="A106" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="B106" s="16" t="s">
+      <c r="B106" s="19" t="s">
         <v>51</v>
       </c>
       <c r="C106" s="17"/>
@@ -2176,7 +2116,7 @@
       <c r="A107" s="12" t="s">
         <v>52</v>
       </c>
-      <c r="B107" s="16" t="s">
+      <c r="B107" s="19" t="s">
         <v>53</v>
       </c>
       <c r="C107" s="17"/>
@@ -2237,7 +2177,7 @@
       <c r="F112" s="4"/>
     </row>
     <row r="113" spans="1:6" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A113" s="24" t="s">
+      <c r="A113" s="22" t="s">
         <v>58</v>
       </c>
       <c r="B113" s="17"/>
@@ -2250,7 +2190,7 @@
       <c r="A114" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="B114" s="16" t="s">
+      <c r="B114" s="19" t="s">
         <v>49</v>
       </c>
       <c r="C114" s="17"/>
@@ -2262,7 +2202,7 @@
       <c r="A115" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="B115" s="16" t="s">
+      <c r="B115" s="19" t="s">
         <v>51</v>
       </c>
       <c r="C115" s="17"/>
@@ -2274,7 +2214,7 @@
       <c r="A116" s="12" t="s">
         <v>52</v>
       </c>
-      <c r="B116" s="16" t="s">
+      <c r="B116" s="19" t="s">
         <v>53</v>
       </c>
       <c r="C116" s="17"/>
@@ -2335,7 +2275,7 @@
       <c r="F121" s="4"/>
     </row>
     <row r="122" spans="1:6" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A122" s="24" t="s">
+      <c r="A122" s="22" t="s">
         <v>59</v>
       </c>
       <c r="B122" s="17"/>
@@ -2348,7 +2288,7 @@
       <c r="A123" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="B123" s="16" t="s">
+      <c r="B123" s="19" t="s">
         <v>49</v>
       </c>
       <c r="C123" s="17"/>
@@ -2360,7 +2300,7 @@
       <c r="A124" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="B124" s="16" t="s">
+      <c r="B124" s="19" t="s">
         <v>51</v>
       </c>
       <c r="C124" s="17"/>
@@ -2372,7 +2312,7 @@
       <c r="A125" s="12" t="s">
         <v>52</v>
       </c>
-      <c r="B125" s="16" t="s">
+      <c r="B125" s="19" t="s">
         <v>53</v>
       </c>
       <c r="C125" s="17"/>
@@ -2433,7 +2373,7 @@
       <c r="F130" s="4"/>
     </row>
     <row r="131" spans="1:6" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A131" s="24" t="s">
+      <c r="A131" s="22" t="s">
         <v>60</v>
       </c>
       <c r="B131" s="17"/>
@@ -2446,7 +2386,7 @@
       <c r="A132" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="B132" s="16" t="s">
+      <c r="B132" s="19" t="s">
         <v>49</v>
       </c>
       <c r="C132" s="17"/>
@@ -2458,7 +2398,7 @@
       <c r="A133" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="B133" s="16" t="s">
+      <c r="B133" s="19" t="s">
         <v>51</v>
       </c>
       <c r="C133" s="17"/>
@@ -2470,7 +2410,7 @@
       <c r="A134" s="12" t="s">
         <v>52</v>
       </c>
-      <c r="B134" s="16" t="s">
+      <c r="B134" s="19" t="s">
         <v>53</v>
       </c>
       <c r="C134" s="17"/>
@@ -2531,7 +2471,7 @@
       <c r="F139" s="4"/>
     </row>
     <row r="140" spans="1:6" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A140" s="24" t="s">
+      <c r="A140" s="22" t="s">
         <v>61</v>
       </c>
       <c r="B140" s="17"/>
@@ -2544,7 +2484,7 @@
       <c r="A141" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="B141" s="16" t="s">
+      <c r="B141" s="19" t="s">
         <v>49</v>
       </c>
       <c r="C141" s="17"/>
@@ -2556,7 +2496,7 @@
       <c r="A142" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="B142" s="16" t="s">
+      <c r="B142" s="19" t="s">
         <v>51</v>
       </c>
       <c r="C142" s="17"/>
@@ -2568,7 +2508,7 @@
       <c r="A143" s="12" t="s">
         <v>52</v>
       </c>
-      <c r="B143" s="16" t="s">
+      <c r="B143" s="19" t="s">
         <v>53</v>
       </c>
       <c r="C143" s="17"/>
@@ -2629,7 +2569,7 @@
       <c r="F148" s="4"/>
     </row>
     <row r="149" spans="1:6" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A149" s="24" t="s">
+      <c r="A149" s="22" t="s">
         <v>62</v>
       </c>
       <c r="B149" s="17"/>
@@ -2642,7 +2582,7 @@
       <c r="A150" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="B150" s="16" t="s">
+      <c r="B150" s="19" t="s">
         <v>49</v>
       </c>
       <c r="C150" s="17"/>
@@ -2654,7 +2594,7 @@
       <c r="A151" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="B151" s="16" t="s">
+      <c r="B151" s="19" t="s">
         <v>51</v>
       </c>
       <c r="C151" s="17"/>
@@ -2666,7 +2606,7 @@
       <c r="A152" s="12" t="s">
         <v>52</v>
       </c>
-      <c r="B152" s="16" t="s">
+      <c r="B152" s="19" t="s">
         <v>53</v>
       </c>
       <c r="C152" s="17"/>
@@ -2727,7 +2667,7 @@
       <c r="F157" s="4"/>
     </row>
     <row r="158" spans="1:6" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A158" s="24" t="s">
+      <c r="A158" s="22" t="s">
         <v>63</v>
       </c>
       <c r="B158" s="17"/>
@@ -2740,7 +2680,7 @@
       <c r="A159" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="B159" s="16" t="s">
+      <c r="B159" s="19" t="s">
         <v>49</v>
       </c>
       <c r="C159" s="17"/>
@@ -2752,7 +2692,7 @@
       <c r="A160" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="B160" s="16" t="s">
+      <c r="B160" s="19" t="s">
         <v>51</v>
       </c>
       <c r="C160" s="17"/>
@@ -2764,7 +2704,7 @@
       <c r="A161" s="12" t="s">
         <v>52</v>
       </c>
-      <c r="B161" s="16" t="s">
+      <c r="B161" s="19" t="s">
         <v>53</v>
       </c>
       <c r="C161" s="17"/>
@@ -2836,16 +2776,16 @@
       <c r="A168" s="23" t="s">
         <v>64</v>
       </c>
-      <c r="B168" s="20"/>
-      <c r="C168" s="20"/>
-      <c r="D168" s="20"/>
-      <c r="E168" s="21"/>
+      <c r="B168" s="24"/>
+      <c r="C168" s="24"/>
+      <c r="D168" s="24"/>
+      <c r="E168" s="25"/>
       <c r="F168" s="14" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="169" spans="1:6" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A169" s="25" t="s">
+      <c r="A169" s="30" t="s">
         <v>65</v>
       </c>
       <c r="B169" s="17"/>
@@ -2963,14 +2903,14 @@
       <c r="F181" s="4"/>
     </row>
     <row r="182" spans="1:6" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A182" s="19" t="s">
+      <c r="A182" s="33" t="s">
         <v>67</v>
       </c>
-      <c r="B182" s="20"/>
-      <c r="C182" s="20"/>
-      <c r="D182" s="20"/>
-      <c r="E182" s="20"/>
-      <c r="F182" s="21"/>
+      <c r="B182" s="24"/>
+      <c r="C182" s="24"/>
+      <c r="D182" s="24"/>
+      <c r="E182" s="24"/>
+      <c r="F182" s="25"/>
     </row>
     <row r="183" spans="1:6" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A183" s="6" t="s">
@@ -3041,14 +2981,14 @@
       <c r="F189" s="4"/>
     </row>
     <row r="190" spans="1:6" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A190" s="19" t="s">
+      <c r="A190" s="33" t="s">
         <v>74</v>
       </c>
-      <c r="B190" s="20"/>
-      <c r="C190" s="20"/>
-      <c r="D190" s="20"/>
-      <c r="E190" s="20"/>
-      <c r="F190" s="21"/>
+      <c r="B190" s="24"/>
+      <c r="C190" s="24"/>
+      <c r="D190" s="24"/>
+      <c r="E190" s="24"/>
+      <c r="F190" s="25"/>
     </row>
     <row r="191" spans="1:6" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A191" s="6" t="s">
@@ -3145,14 +3085,14 @@
       <c r="F201" s="9"/>
     </row>
     <row r="202" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A202" s="29" t="s">
+      <c r="A202" s="20" t="s">
         <v>78</v>
       </c>
       <c r="B202" s="10" t="str">
         <f>IFERROR(AVERAGE(B192:B197),"")</f>
         <v/>
       </c>
-      <c r="C202" s="30"/>
+      <c r="C202" s="34"/>
       <c r="D202" s="17"/>
       <c r="E202" s="17"/>
       <c r="F202" s="18"/>
@@ -3177,6 +3117,64 @@
     </row>
   </sheetData>
   <mergeCells count="74">
+    <mergeCell ref="B125:F125"/>
+    <mergeCell ref="B105:F105"/>
+    <mergeCell ref="B143:F143"/>
+    <mergeCell ref="A182:F182"/>
+    <mergeCell ref="A45:F45"/>
+    <mergeCell ref="B133:F133"/>
+    <mergeCell ref="A168:E168"/>
+    <mergeCell ref="A158:F158"/>
+    <mergeCell ref="B161:F161"/>
+    <mergeCell ref="A169:F169"/>
+    <mergeCell ref="B142:F142"/>
+    <mergeCell ref="E54:F54"/>
+    <mergeCell ref="B80:F80"/>
+    <mergeCell ref="B124:F124"/>
+    <mergeCell ref="B89:F89"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="A44:E44"/>
+    <mergeCell ref="A104:F104"/>
+    <mergeCell ref="A55:F55"/>
+    <mergeCell ref="B114:F114"/>
+    <mergeCell ref="A21:F21"/>
+    <mergeCell ref="B106:F106"/>
+    <mergeCell ref="A95:F95"/>
+    <mergeCell ref="B87:F87"/>
+    <mergeCell ref="A11:E11"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="A202"/>
+    <mergeCell ref="A86:F86"/>
+    <mergeCell ref="C202:F202"/>
+    <mergeCell ref="E3:F3"/>
+    <mergeCell ref="A32:F32"/>
+    <mergeCell ref="B151:F151"/>
+    <mergeCell ref="B96:F96"/>
+    <mergeCell ref="B116:F116"/>
+    <mergeCell ref="B160:F160"/>
+    <mergeCell ref="A6:E6"/>
+    <mergeCell ref="A149:F149"/>
+    <mergeCell ref="B150:F150"/>
+    <mergeCell ref="A7:F7"/>
+    <mergeCell ref="B97:F97"/>
+    <mergeCell ref="A140:F140"/>
+    <mergeCell ref="A23:E23"/>
+    <mergeCell ref="A204:F204"/>
+    <mergeCell ref="A34:E34"/>
+    <mergeCell ref="A190:F190"/>
+    <mergeCell ref="B152:F152"/>
+    <mergeCell ref="A35:F35"/>
+    <mergeCell ref="A122:F122"/>
+    <mergeCell ref="B132:F132"/>
+    <mergeCell ref="A131:F131"/>
+    <mergeCell ref="B141:F141"/>
+    <mergeCell ref="B159:F159"/>
+    <mergeCell ref="B134:F134"/>
+    <mergeCell ref="B115:F115"/>
+    <mergeCell ref="B107:F107"/>
+    <mergeCell ref="B98:F98"/>
+    <mergeCell ref="A76:F76"/>
+    <mergeCell ref="A113:F113"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="B88:F88"/>
     <mergeCell ref="B123:F123"/>
@@ -3193,64 +3191,6 @@
     <mergeCell ref="A12:F12"/>
     <mergeCell ref="A58:F58"/>
     <mergeCell ref="B2:C2"/>
-    <mergeCell ref="A204:F204"/>
-    <mergeCell ref="A34:E34"/>
-    <mergeCell ref="A190:F190"/>
-    <mergeCell ref="B152:F152"/>
-    <mergeCell ref="A35:F35"/>
-    <mergeCell ref="A122:F122"/>
-    <mergeCell ref="B132:F132"/>
-    <mergeCell ref="A131:F131"/>
-    <mergeCell ref="B141:F141"/>
-    <mergeCell ref="B159:F159"/>
-    <mergeCell ref="B134:F134"/>
-    <mergeCell ref="B115:F115"/>
-    <mergeCell ref="B107:F107"/>
-    <mergeCell ref="B98:F98"/>
-    <mergeCell ref="A76:F76"/>
-    <mergeCell ref="A113:F113"/>
-    <mergeCell ref="A202"/>
-    <mergeCell ref="A86:F86"/>
-    <mergeCell ref="C202:F202"/>
-    <mergeCell ref="E3:F3"/>
-    <mergeCell ref="A32:F32"/>
-    <mergeCell ref="B151:F151"/>
-    <mergeCell ref="B96:F96"/>
-    <mergeCell ref="B116:F116"/>
-    <mergeCell ref="B160:F160"/>
-    <mergeCell ref="A6:E6"/>
-    <mergeCell ref="A149:F149"/>
-    <mergeCell ref="B150:F150"/>
-    <mergeCell ref="A7:F7"/>
-    <mergeCell ref="B97:F97"/>
-    <mergeCell ref="A140:F140"/>
-    <mergeCell ref="A23:E23"/>
-    <mergeCell ref="E4:F4"/>
-    <mergeCell ref="A44:E44"/>
-    <mergeCell ref="A104:F104"/>
-    <mergeCell ref="A55:F55"/>
-    <mergeCell ref="B114:F114"/>
-    <mergeCell ref="A21:F21"/>
-    <mergeCell ref="B106:F106"/>
-    <mergeCell ref="A95:F95"/>
-    <mergeCell ref="B87:F87"/>
-    <mergeCell ref="A11:E11"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="B125:F125"/>
-    <mergeCell ref="B105:F105"/>
-    <mergeCell ref="B143:F143"/>
-    <mergeCell ref="A182:F182"/>
-    <mergeCell ref="A45:F45"/>
-    <mergeCell ref="B133:F133"/>
-    <mergeCell ref="A168:E168"/>
-    <mergeCell ref="A158:F158"/>
-    <mergeCell ref="B161:F161"/>
-    <mergeCell ref="A169:F169"/>
-    <mergeCell ref="B142:F142"/>
-    <mergeCell ref="E54:F54"/>
-    <mergeCell ref="B80:F80"/>
-    <mergeCell ref="B124:F124"/>
-    <mergeCell ref="B89:F89"/>
   </mergeCells>
   <dataValidations count="9">
     <dataValidation type="list" allowBlank="1" sqref="E14:E20" xr:uid="{00000000-0002-0000-0000-000000000000}">
@@ -3297,7 +3237,7 @@
   <sheetData>
     <row r="1" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="39" t="s">
-        <v>123</v>
+        <v>103</v>
       </c>
       <c r="B1" s="17"/>
       <c r="C1" s="17"/>
@@ -3371,9 +3311,7 @@
       </c>
     </row>
     <row r="4" spans="1:13" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="13" t="s">
-        <v>115</v>
-      </c>
+      <c r="A4" s="13"/>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
@@ -3388,9 +3326,7 @@
       <c r="M4" s="3"/>
     </row>
     <row r="5" spans="1:13" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="13" t="s">
-        <v>116</v>
-      </c>
+      <c r="A5" s="13"/>
       <c r="B5" s="9"/>
       <c r="C5" s="9"/>
       <c r="D5" s="9"/>
@@ -3405,9 +3341,7 @@
       <c r="M5" s="9"/>
     </row>
     <row r="6" spans="1:13" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="13" t="s">
-        <v>117</v>
-      </c>
+      <c r="A6" s="13"/>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
@@ -3422,9 +3356,7 @@
       <c r="M6" s="3"/>
     </row>
     <row r="7" spans="1:13" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="13" t="s">
-        <v>118</v>
-      </c>
+      <c r="A7" s="13"/>
       <c r="B7" s="9"/>
       <c r="C7" s="9"/>
       <c r="D7" s="9"/>
@@ -3439,9 +3371,7 @@
       <c r="M7" s="9"/>
     </row>
     <row r="8" spans="1:13" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="2" t="s">
-        <v>92</v>
-      </c>
+      <c r="A8" s="2"/>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
       <c r="D8" s="3"/>
@@ -3456,9 +3386,7 @@
       <c r="M8" s="3"/>
     </row>
     <row r="9" spans="1:13" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="8" t="s">
-        <v>93</v>
-      </c>
+      <c r="A9" s="8"/>
       <c r="B9" s="9"/>
       <c r="C9" s="9"/>
       <c r="D9" s="9"/>
@@ -3473,9 +3401,7 @@
       <c r="M9" s="9"/>
     </row>
     <row r="10" spans="1:13" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="2" t="s">
-        <v>94</v>
-      </c>
+      <c r="A10" s="2"/>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
       <c r="D10" s="3"/>
@@ -3490,9 +3416,7 @@
       <c r="M10" s="3"/>
     </row>
     <row r="11" spans="1:13" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="8" t="s">
-        <v>95</v>
-      </c>
+      <c r="A11" s="8"/>
       <c r="B11" s="9"/>
       <c r="C11" s="9"/>
       <c r="D11" s="9"/>
@@ -3507,9 +3431,7 @@
       <c r="M11" s="9"/>
     </row>
     <row r="12" spans="1:13" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="2" t="s">
-        <v>96</v>
-      </c>
+      <c r="A12" s="2"/>
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
       <c r="D12" s="3"/>
@@ -3524,9 +3446,7 @@
       <c r="M12" s="3"/>
     </row>
     <row r="13" spans="1:13" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="8" t="s">
-        <v>97</v>
-      </c>
+      <c r="A13" s="8"/>
       <c r="B13" s="9"/>
       <c r="C13" s="9"/>
       <c r="D13" s="9"/>
@@ -3557,7 +3477,7 @@
     </row>
     <row r="15" spans="1:13" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="37" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="B15" s="32"/>
       <c r="C15" s="32"/>
@@ -3598,7 +3518,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="39" t="s">
-        <v>124</v>
+        <v>104</v>
       </c>
       <c r="B1" s="17"/>
       <c r="C1" s="17"/>
@@ -3610,7 +3530,7 @@
     </row>
     <row r="2" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="41" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="B2" s="17"/>
       <c r="C2" s="17"/>
@@ -3621,8 +3541,8 @@
       <c r="H2" s="18"/>
     </row>
     <row r="3" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="22" t="s">
-        <v>100</v>
+      <c r="A3" s="26" t="s">
+        <v>94</v>
       </c>
       <c r="B3" s="17"/>
       <c r="C3" s="17"/>
@@ -3634,7 +3554,7 @@
     </row>
     <row r="4" spans="1:8" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="B4" s="11" t="s">
         <v>22</v>
@@ -3662,9 +3582,7 @@
       <c r="A5" s="3">
         <v>1</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>102</v>
-      </c>
+      <c r="B5" s="2"/>
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
       <c r="E5" s="3"/>
@@ -3676,9 +3594,7 @@
       <c r="A6" s="9">
         <v>2</v>
       </c>
-      <c r="B6" s="8" t="s">
-        <v>103</v>
-      </c>
+      <c r="B6" s="8"/>
       <c r="C6" s="9"/>
       <c r="D6" s="9"/>
       <c r="E6" s="9"/>
@@ -3690,9 +3606,7 @@
       <c r="A7" s="3">
         <v>3</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>104</v>
-      </c>
+      <c r="B7" s="2"/>
       <c r="C7" s="3"/>
       <c r="D7" s="3"/>
       <c r="E7" s="3"/>
@@ -3704,9 +3618,7 @@
       <c r="A8" s="9">
         <v>4</v>
       </c>
-      <c r="B8" s="8" t="s">
-        <v>105</v>
-      </c>
+      <c r="B8" s="8"/>
       <c r="C8" s="9"/>
       <c r="D8" s="9"/>
       <c r="E8" s="9"/>
@@ -3718,9 +3630,7 @@
       <c r="A9" s="3">
         <v>5</v>
       </c>
-      <c r="B9" s="2" t="s">
-        <v>106</v>
-      </c>
+      <c r="B9" s="2"/>
       <c r="C9" s="3"/>
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
@@ -3732,9 +3642,7 @@
       <c r="A10" s="9">
         <v>6</v>
       </c>
-      <c r="B10" s="8" t="s">
-        <v>107</v>
-      </c>
+      <c r="B10" s="8"/>
       <c r="C10" s="9"/>
       <c r="D10" s="9"/>
       <c r="E10" s="9"/>
@@ -3746,9 +3654,7 @@
       <c r="A11" s="3">
         <v>7</v>
       </c>
-      <c r="B11" s="2" t="s">
-        <v>108</v>
-      </c>
+      <c r="B11" s="2"/>
       <c r="C11" s="3"/>
       <c r="D11" s="3"/>
       <c r="E11" s="3"/>
@@ -3760,9 +3666,7 @@
       <c r="A12" s="9">
         <v>8</v>
       </c>
-      <c r="B12" s="13" t="s">
-        <v>119</v>
-      </c>
+      <c r="B12" s="13"/>
       <c r="C12" s="9"/>
       <c r="D12" s="9"/>
       <c r="E12" s="9"/>
@@ -3774,9 +3678,7 @@
       <c r="A13" s="3">
         <v>9</v>
       </c>
-      <c r="B13" s="13" t="s">
-        <v>120</v>
-      </c>
+      <c r="B13" s="13"/>
       <c r="C13" s="3"/>
       <c r="D13" s="3"/>
       <c r="E13" s="3"/>
@@ -3788,9 +3690,7 @@
       <c r="A14" s="9">
         <v>10</v>
       </c>
-      <c r="B14" s="13" t="s">
-        <v>121</v>
-      </c>
+      <c r="B14" s="13"/>
       <c r="C14" s="9"/>
       <c r="D14" s="9"/>
       <c r="E14" s="9"/>
@@ -3809,8 +3709,8 @@
       <c r="H15" s="4"/>
     </row>
     <row r="16" spans="1:8" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="25" t="s">
-        <v>109</v>
+      <c r="A16" s="30" t="s">
+        <v>96</v>
       </c>
       <c r="B16" s="17"/>
       <c r="C16" s="17"/>
@@ -3822,7 +3722,7 @@
     </row>
     <row r="17" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="40" t="s">
-        <v>110</v>
+        <v>97</v>
       </c>
       <c r="B17" s="17"/>
       <c r="C17" s="17"/>
@@ -3834,16 +3734,16 @@
     </row>
     <row r="18" spans="1:8" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="7" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>111</v>
+        <v>98</v>
       </c>
       <c r="C18" s="7" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>112</v>
+        <v>99</v>
       </c>
       <c r="E18" s="7" t="s">
         <v>16</v>
@@ -3906,7 +3806,7 @@
     </row>
     <row r="23" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="40" t="s">
-        <v>113</v>
+        <v>100</v>
       </c>
       <c r="B23" s="17"/>
       <c r="C23" s="17"/>
@@ -3918,16 +3818,16 @@
     </row>
     <row r="24" spans="1:8" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="7" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>111</v>
+        <v>98</v>
       </c>
       <c r="C24" s="7" t="s">
         <v>14</v>
       </c>
       <c r="D24" s="7" t="s">
-        <v>112</v>
+        <v>99</v>
       </c>
       <c r="E24" s="7" t="s">
         <v>16</v>
@@ -3990,7 +3890,7 @@
     </row>
     <row r="29" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="40" t="s">
-        <v>114</v>
+        <v>101</v>
       </c>
       <c r="B29" s="17"/>
       <c r="C29" s="17"/>
@@ -4002,16 +3902,16 @@
     </row>
     <row r="30" spans="1:8" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="7" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>111</v>
+        <v>98</v>
       </c>
       <c r="C30" s="7" t="s">
         <v>14</v>
       </c>
       <c r="D30" s="7" t="s">
-        <v>112</v>
+        <v>99</v>
       </c>
       <c r="E30" s="7" t="s">
         <v>16</v>
@@ -4087,12 +3987,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0df7f343-3985-4f2e-a59f-0a9fbfed1bd2">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b5d7b36e-83e1-4fd4-8dab-8bf7437cf9c0" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4347,20 +4249,29 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0df7f343-3985-4f2e-a59f-0a9fbfed1bd2">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b5d7b36e-83e1-4fd4-8dab-8bf7437cf9c0" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FCBA2542-ED56-4814-A955-A834AC10978F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7B8B28E6-E08A-4A50-B2CC-8A0D8DF4030B}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="90c00910-8be4-4468-a61a-5db5f02684d1"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="b5d7b36e-83e1-4fd4-8dab-8bf7437cf9c0"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="0df7f343-3985-4f2e-a59f-0a9fbfed1bd2"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="309133ba-e894-457a-a252-d76c370bc267"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -4387,20 +4298,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7B8B28E6-E08A-4A50-B2CC-8A0D8DF4030B}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FCBA2542-ED56-4814-A955-A834AC10978F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="90c00910-8be4-4468-a61a-5db5f02684d1"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="b5d7b36e-83e1-4fd4-8dab-8bf7437cf9c0"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="0df7f343-3985-4f2e-a59f-0a9fbfed1bd2"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="309133ba-e894-457a-a252-d76c370bc267"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>